<commit_message>
TBCP: add 14 cross-referenced schedules (S1-S14)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NhaKeVxjNyTBn6poC6zJrZ
</commit_message>
<xml_diff>
--- a/Lumbee_RIVR_TBCP_Agreement_Package/05_Schedules/S8_Subscriber_Payment_Revenue_ProgramIncome_Tax_Audit.xlsx
+++ b/Lumbee_RIVR_TBCP_Agreement_Package/05_Schedules/S8_Subscriber_Payment_Revenue_ProgramIncome_Tax_Audit.xlsx
@@ -1404,9 +1404,10 @@
         <f>IF(AND(ISNUMBER(B6),ISNUMBER(B7)),B6*B7,"")</f>
         <v/>
       </c>
-      <c r="C8" s="14">
-        <f> Subscribers x Rate</f>
-        <v/>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>Subscribers x Rate</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -1419,9 +1420,10 @@
         <f>IF(ISNUMBER(B8),B8*12,"")</f>
         <v/>
       </c>
-      <c r="C9" s="14">
-        <f> Monthly x 12</f>
-        <v/>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>Monthly x 12</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>